<commit_message>
feat(resource): intake Aug water/energy and refresh GHG provenance
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data/staging/source/1.1Water.xlsx
+++ b/data/staging/source/1.1Water.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30417"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30425"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://maejo365-my.sharepoint.com/personal/researchmju_mju_ac_th/Documents/RAE-Document-Center/07-GreenOffice/resource/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="8" documentId="8_{68807AFC-3756-48AE-906F-0C299039043D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C1CD58F2-709F-4FC7-BDA5-141DC454637F}"/>
+  <xr:revisionPtr revIDLastSave="10" documentId="8_{68807AFC-3756-48AE-906F-0C299039043D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FBFF9B8C-DCE7-4AD7-8CAD-3C7890D5A8EF}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13140" xr2:uid="{3D263492-E412-45DB-BC97-661FEC5BE144}"/>
   </bookViews>
@@ -1017,9 +1017,6 @@
     <xf numFmtId="0" fontId="16" fillId="2" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1035,34 +1032,10 @@
     <xf numFmtId="0" fontId="13" fillId="4" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="6" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1079,6 +1052,33 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -1406,7 +1406,7 @@
                   <c:v>646.3599999999999</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>-2409.5</c:v>
+                  <c:v>592.90999999999985</c:v>
                 </c:pt>
                 <c:pt idx="8">
                   <c:v>0</c:v>
@@ -1421,7 +1421,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>263.54416666666663</c:v>
+                  <c:v>513.745</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3242,7 +3242,7 @@
                   <c:v>6.8761702127659561</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>-25.632978723404257</c:v>
+                  <c:v>6.3075531914893599</c:v>
                 </c:pt>
                 <c:pt idx="8">
                   <c:v>0</c:v>
@@ -3257,7 +3257,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>2.8036613475177301</c:v>
+                  <c:v>5.4653723404255317</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3690,7 +3690,7 @@
                   <c:v>8337.5</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>3162.5299999999997</c:v>
+                  <c:v>6164.94</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4043,7 +4043,7 @@
                   <c:v>8.4195273265744142</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>33.643936170212761</c:v>
+                  <c:v>65.58446808510638</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -12512,7 +12512,7 @@
     <col min="16139" max="16384" width="9" style="31"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" ht="21.75" customHeight="1">
+    <row r="1" spans="1:16" ht="21.75" customHeight="1">
       <c r="A1" s="29"/>
       <c r="B1" s="30"/>
       <c r="C1" s="30"/>
@@ -12527,42 +12527,42 @@
       </c>
       <c r="L1" s="30"/>
     </row>
-    <row r="2" spans="1:19" ht="23.1" customHeight="1" thickBot="1">
-      <c r="A2" s="73" t="s">
+    <row r="2" spans="1:16" ht="23.1" customHeight="1" thickBot="1">
+      <c r="A2" s="72" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="73"/>
-      <c r="C2" s="73"/>
-      <c r="D2" s="73"/>
-      <c r="E2" s="73"/>
-      <c r="F2" s="73"/>
-      <c r="G2" s="73"/>
-      <c r="H2" s="73"/>
-      <c r="I2" s="73"/>
-      <c r="J2" s="73"/>
-      <c r="K2" s="73"/>
+      <c r="B2" s="72"/>
+      <c r="C2" s="72"/>
+      <c r="D2" s="72"/>
+      <c r="E2" s="72"/>
+      <c r="F2" s="72"/>
+      <c r="G2" s="72"/>
+      <c r="H2" s="72"/>
+      <c r="I2" s="72"/>
+      <c r="J2" s="72"/>
+      <c r="K2" s="72"/>
       <c r="L2" s="30"/>
     </row>
-    <row r="3" spans="1:19" s="34" customFormat="1" ht="21.6" customHeight="1">
-      <c r="A3" s="74" t="s">
+    <row r="3" spans="1:16" s="34" customFormat="1" ht="21.6" customHeight="1">
+      <c r="A3" s="73" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="75" t="s">
+      <c r="B3" s="74" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="75"/>
-      <c r="D3" s="75"/>
-      <c r="E3" s="75"/>
-      <c r="F3" s="75" t="s">
+      <c r="C3" s="74"/>
+      <c r="D3" s="74"/>
+      <c r="E3" s="74"/>
+      <c r="F3" s="74" t="s">
         <v>4</v>
       </c>
-      <c r="G3" s="75"/>
-      <c r="H3" s="75"/>
-      <c r="I3" s="75"/>
-      <c r="J3" s="75" t="s">
+      <c r="G3" s="74"/>
+      <c r="H3" s="74"/>
+      <c r="I3" s="74"/>
+      <c r="J3" s="74" t="s">
         <v>5</v>
       </c>
-      <c r="K3" s="75"/>
+      <c r="K3" s="74"/>
       <c r="M3" s="35" t="s">
         <v>6</v>
       </c>
@@ -12570,8 +12570,8 @@
       <c r="O3" s="36"/>
       <c r="P3" s="37"/>
     </row>
-    <row r="4" spans="1:19" s="34" customFormat="1" ht="45.95" customHeight="1">
-      <c r="A4" s="74"/>
+    <row r="4" spans="1:16" s="34" customFormat="1" ht="45.95" customHeight="1">
+      <c r="A4" s="73"/>
       <c r="B4" s="33" t="s">
         <v>7</v>
       </c>
@@ -12613,7 +12613,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:19" ht="24.95" customHeight="1">
+    <row r="5" spans="1:16" ht="24.95" customHeight="1">
       <c r="A5" s="41" t="s">
         <v>18</v>
       </c>
@@ -12669,7 +12669,7 @@
         <v>1098.4000000000233</v>
       </c>
     </row>
-    <row r="6" spans="1:19" ht="24.95" customHeight="1">
+    <row r="6" spans="1:16" ht="24.95" customHeight="1">
       <c r="A6" s="41" t="s">
         <v>20</v>
       </c>
@@ -12725,7 +12725,7 @@
         <v>944.59999999997672</v>
       </c>
     </row>
-    <row r="7" spans="1:19" ht="24.95" customHeight="1">
+    <row r="7" spans="1:16" ht="24.95" customHeight="1">
       <c r="A7" s="41" t="s">
         <v>22</v>
       </c>
@@ -12780,11 +12780,8 @@
         <f t="shared" si="7"/>
         <v>909.70000000001164</v>
       </c>
-      <c r="S7" s="31">
-        <v>288740.5</v>
-      </c>
     </row>
-    <row r="8" spans="1:19" ht="24.95" customHeight="1">
+    <row r="8" spans="1:16" ht="24.95" customHeight="1">
       <c r="A8" s="41" t="s">
         <v>24</v>
       </c>
@@ -12840,7 +12837,7 @@
         <v>858.29999999998836</v>
       </c>
     </row>
-    <row r="9" spans="1:19" ht="24.95" customHeight="1">
+    <row r="9" spans="1:16" ht="24.95" customHeight="1">
       <c r="A9" s="41" t="s">
         <v>26</v>
       </c>
@@ -12896,7 +12893,7 @@
         <v>539.96</v>
       </c>
     </row>
-    <row r="10" spans="1:19" ht="24.95" customHeight="1">
+    <row r="10" spans="1:16" ht="24.95" customHeight="1">
       <c r="A10" s="41" t="s">
         <v>28</v>
       </c>
@@ -12952,7 +12949,7 @@
         <v>574.71</v>
       </c>
     </row>
-    <row r="11" spans="1:19" ht="24.95" customHeight="1">
+    <row r="11" spans="1:16" ht="24.95" customHeight="1">
       <c r="A11" s="41" t="s">
         <v>30</v>
       </c>
@@ -13008,7 +13005,7 @@
         <v>646.3599999999999</v>
       </c>
     </row>
-    <row r="12" spans="1:19" ht="24.95" customHeight="1">
+    <row r="12" spans="1:16" ht="24.95" customHeight="1">
       <c r="A12" s="41" t="s">
         <v>32</v>
       </c>
@@ -13032,37 +13029,39 @@
       </c>
       <c r="G12" s="44">
         <f t="shared" si="2"/>
-        <v>-2409.5</v>
+        <v>592.90999999999985</v>
       </c>
       <c r="H12" s="43">
         <f t="shared" si="3"/>
-        <v>-19276</v>
+        <v>4743.2799999999988</v>
       </c>
       <c r="I12" s="43">
         <f t="shared" si="4"/>
-        <v>-25.632978723404257</v>
+        <v>6.3075531914893599</v>
       </c>
       <c r="J12" s="14">
         <f t="shared" si="5"/>
-        <v>-4.4594400574300073</v>
+        <v>-0.14872936109117035</v>
       </c>
       <c r="K12" s="15">
         <f t="shared" si="6"/>
-        <v>-51.603511478364467</v>
+        <v>11.452097111698306</v>
       </c>
       <c r="M12" s="45" t="s">
         <v>33</v>
       </c>
-      <c r="N12" s="47"/>
+      <c r="N12" s="47">
+        <v>3002.41</v>
+      </c>
       <c r="O12" s="47">
         <v>2409.5</v>
       </c>
       <c r="P12" s="48">
         <f t="shared" si="7"/>
-        <v>-2409.5</v>
+        <v>592.90999999999985</v>
       </c>
     </row>
-    <row r="13" spans="1:19" ht="24.95" customHeight="1">
+    <row r="13" spans="1:16" ht="24.95" customHeight="1">
       <c r="A13" s="41" t="s">
         <v>34</v>
       </c>
@@ -13114,7 +13113,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:19" ht="24.95" customHeight="1">
+    <row r="14" spans="1:16" ht="24.95" customHeight="1">
       <c r="A14" s="41" t="s">
         <v>36</v>
       </c>
@@ -13166,7 +13165,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:19" ht="24.95" customHeight="1">
+    <row r="15" spans="1:16" ht="24.95" customHeight="1">
       <c r="A15" s="41" t="s">
         <v>38</v>
       </c>
@@ -13218,7 +13217,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:19" ht="24.95" customHeight="1" thickBot="1">
+    <row r="16" spans="1:16" ht="24.95" customHeight="1" thickBot="1">
       <c r="A16" s="41" t="s">
         <v>40</v>
       </c>
@@ -13296,23 +13295,23 @@
       </c>
       <c r="G17" s="43">
         <f t="shared" si="8"/>
-        <v>263.54416666666663</v>
+        <v>513.745</v>
       </c>
       <c r="H17" s="43">
         <f t="shared" si="8"/>
-        <v>2108.353333333333</v>
+        <v>4109.96</v>
       </c>
       <c r="I17" s="43">
         <f>G17/F17</f>
-        <v>2.8036613475177301</v>
+        <v>5.4653723404255317</v>
       </c>
       <c r="J17" s="14">
         <f>(G17-C17)/C17</f>
-        <v>-0.62068605697151424</v>
+        <v>-0.26057691154422785</v>
       </c>
       <c r="K17" s="15">
         <f>(I17-E17)/E17</f>
-        <v>2.9959412049204901</v>
+        <v>6.7895665090489361</v>
       </c>
     </row>
     <row r="18" spans="1:11" ht="24.95" customHeight="1">
@@ -13341,23 +13340,23 @@
       </c>
       <c r="G18" s="43">
         <f t="shared" si="9"/>
-        <v>3162.5299999999997</v>
+        <v>6164.94</v>
       </c>
       <c r="H18" s="43">
         <f t="shared" si="9"/>
-        <v>25300.239999999998</v>
+        <v>49319.519999999997</v>
       </c>
       <c r="I18" s="43">
         <f t="shared" si="9"/>
-        <v>33.643936170212761</v>
+        <v>65.58446808510638</v>
       </c>
       <c r="J18" s="14">
         <f t="shared" si="5"/>
-        <v>-0.62068605697151424</v>
+        <v>-0.26057691154422791</v>
       </c>
       <c r="K18" s="15">
         <f t="shared" si="6"/>
-        <v>2.9959412049204905</v>
+        <v>6.7895665090489361</v>
       </c>
     </row>
     <row r="19" spans="1:11" ht="11.45" customHeight="1">
@@ -13401,76 +13400,76 @@
     </row>
     <row r="40" spans="1:12" ht="21.95" customHeight="1"/>
     <row r="43" spans="1:12" ht="21.75" customHeight="1">
-      <c r="A43" s="76" t="s">
+      <c r="A43" s="75" t="s">
         <v>44</v>
       </c>
-      <c r="B43" s="76"/>
-      <c r="C43" s="76"/>
-      <c r="D43" s="76"/>
-      <c r="E43" s="76"/>
-      <c r="F43" s="76"/>
-      <c r="G43" s="76"/>
-      <c r="H43" s="76"/>
-      <c r="I43" s="76"/>
-      <c r="J43" s="76"/>
-      <c r="K43" s="76"/>
-      <c r="L43" s="76"/>
+      <c r="B43" s="75"/>
+      <c r="C43" s="75"/>
+      <c r="D43" s="75"/>
+      <c r="E43" s="75"/>
+      <c r="F43" s="75"/>
+      <c r="G43" s="75"/>
+      <c r="H43" s="75"/>
+      <c r="I43" s="75"/>
+      <c r="J43" s="75"/>
+      <c r="K43" s="75"/>
+      <c r="L43" s="75"/>
     </row>
     <row r="44" spans="1:12" ht="21.75" customHeight="1">
-      <c r="A44" s="76"/>
-      <c r="B44" s="76"/>
-      <c r="C44" s="76"/>
-      <c r="D44" s="76"/>
-      <c r="E44" s="76"/>
-      <c r="F44" s="76"/>
-      <c r="G44" s="76"/>
-      <c r="H44" s="76"/>
-      <c r="I44" s="76"/>
-      <c r="J44" s="76"/>
-      <c r="K44" s="76"/>
-      <c r="L44" s="76"/>
+      <c r="A44" s="75"/>
+      <c r="B44" s="75"/>
+      <c r="C44" s="75"/>
+      <c r="D44" s="75"/>
+      <c r="E44" s="75"/>
+      <c r="F44" s="75"/>
+      <c r="G44" s="75"/>
+      <c r="H44" s="75"/>
+      <c r="I44" s="75"/>
+      <c r="J44" s="75"/>
+      <c r="K44" s="75"/>
+      <c r="L44" s="75"/>
     </row>
     <row r="45" spans="1:12" ht="21.75" customHeight="1">
-      <c r="A45" s="76"/>
-      <c r="B45" s="76"/>
-      <c r="C45" s="76"/>
-      <c r="D45" s="76"/>
-      <c r="E45" s="76"/>
-      <c r="F45" s="76"/>
-      <c r="G45" s="76"/>
-      <c r="H45" s="76"/>
-      <c r="I45" s="76"/>
-      <c r="J45" s="76"/>
-      <c r="K45" s="76"/>
-      <c r="L45" s="76"/>
+      <c r="A45" s="75"/>
+      <c r="B45" s="75"/>
+      <c r="C45" s="75"/>
+      <c r="D45" s="75"/>
+      <c r="E45" s="75"/>
+      <c r="F45" s="75"/>
+      <c r="G45" s="75"/>
+      <c r="H45" s="75"/>
+      <c r="I45" s="75"/>
+      <c r="J45" s="75"/>
+      <c r="K45" s="75"/>
+      <c r="L45" s="75"/>
     </row>
     <row r="46" spans="1:12" ht="21.75" customHeight="1">
-      <c r="A46" s="76"/>
-      <c r="B46" s="76"/>
-      <c r="C46" s="76"/>
-      <c r="D46" s="76"/>
-      <c r="E46" s="76"/>
-      <c r="F46" s="76"/>
-      <c r="G46" s="76"/>
-      <c r="H46" s="76"/>
-      <c r="I46" s="76"/>
-      <c r="J46" s="76"/>
-      <c r="K46" s="76"/>
-      <c r="L46" s="76"/>
+      <c r="A46" s="75"/>
+      <c r="B46" s="75"/>
+      <c r="C46" s="75"/>
+      <c r="D46" s="75"/>
+      <c r="E46" s="75"/>
+      <c r="F46" s="75"/>
+      <c r="G46" s="75"/>
+      <c r="H46" s="75"/>
+      <c r="I46" s="75"/>
+      <c r="J46" s="75"/>
+      <c r="K46" s="75"/>
+      <c r="L46" s="75"/>
     </row>
     <row r="47" spans="1:12" ht="38.450000000000003" customHeight="1">
-      <c r="A47" s="76"/>
-      <c r="B47" s="76"/>
-      <c r="C47" s="76"/>
-      <c r="D47" s="76"/>
-      <c r="E47" s="76"/>
-      <c r="F47" s="76"/>
-      <c r="G47" s="76"/>
-      <c r="H47" s="76"/>
-      <c r="I47" s="76"/>
-      <c r="J47" s="76"/>
-      <c r="K47" s="76"/>
-      <c r="L47" s="76"/>
+      <c r="A47" s="75"/>
+      <c r="B47" s="75"/>
+      <c r="C47" s="75"/>
+      <c r="D47" s="75"/>
+      <c r="E47" s="75"/>
+      <c r="F47" s="75"/>
+      <c r="G47" s="75"/>
+      <c r="H47" s="75"/>
+      <c r="I47" s="75"/>
+      <c r="J47" s="75"/>
+      <c r="K47" s="75"/>
+      <c r="L47" s="75"/>
     </row>
     <row r="48" spans="1:12" s="57" customFormat="1" ht="38.450000000000003" customHeight="1">
       <c r="A48" s="56"/>
@@ -13490,20 +13489,20 @@
       <c r="L48" s="56"/>
     </row>
     <row r="49" spans="1:17" ht="42" customHeight="1">
-      <c r="A49" s="77" t="s">
+      <c r="A49" s="76" t="s">
         <v>47</v>
       </c>
-      <c r="B49" s="77"/>
-      <c r="C49" s="77"/>
-      <c r="D49" s="77"/>
-      <c r="E49" s="77"/>
-      <c r="F49" s="77"/>
-      <c r="G49" s="77"/>
-      <c r="H49" s="77"/>
-      <c r="I49" s="77"/>
-      <c r="J49" s="77"/>
-      <c r="K49" s="77"/>
-      <c r="L49" s="77"/>
+      <c r="B49" s="76"/>
+      <c r="C49" s="76"/>
+      <c r="D49" s="76"/>
+      <c r="E49" s="76"/>
+      <c r="F49" s="76"/>
+      <c r="G49" s="76"/>
+      <c r="H49" s="76"/>
+      <c r="I49" s="76"/>
+      <c r="J49" s="76"/>
+      <c r="K49" s="76"/>
+      <c r="L49" s="76"/>
       <c r="N49" s="59"/>
       <c r="O49" s="60"/>
       <c r="P49" s="61"/>
@@ -13537,10 +13536,10 @@
       <c r="C51" s="65"/>
     </row>
     <row r="52" spans="1:17" s="63" customFormat="1" ht="50.1" customHeight="1">
-      <c r="A52" s="72" t="s">
+      <c r="A52" s="77" t="s">
         <v>50</v>
       </c>
-      <c r="B52" s="72"/>
+      <c r="B52" s="77"/>
       <c r="C52" s="66"/>
       <c r="D52" s="67"/>
     </row>
@@ -13580,10 +13579,10 @@
       <c r="D55" s="64"/>
     </row>
     <row r="56" spans="1:17" s="63" customFormat="1" ht="50.1" customHeight="1">
-      <c r="A56" s="72" t="s">
+      <c r="A56" s="77" t="s">
         <v>50</v>
       </c>
-      <c r="B56" s="72"/>
+      <c r="B56" s="77"/>
       <c r="C56" s="66"/>
       <c r="D56" s="67"/>
     </row>
@@ -13795,10 +13794,10 @@
       <c r="C75" s="65"/>
     </row>
     <row r="76" spans="1:12" s="63" customFormat="1" ht="39.950000000000003" customHeight="1">
-      <c r="A76" s="72" t="s">
+      <c r="A76" s="77" t="s">
         <v>50</v>
       </c>
-      <c r="B76" s="72"/>
+      <c r="B76" s="77"/>
       <c r="C76" s="66"/>
       <c r="D76" s="67"/>
     </row>
@@ -13838,10 +13837,10 @@
       <c r="D79" s="64"/>
     </row>
     <row r="80" spans="1:12" s="63" customFormat="1" ht="39.950000000000003" customHeight="1">
-      <c r="A80" s="72" t="s">
+      <c r="A80" s="77" t="s">
         <v>50</v>
       </c>
-      <c r="B80" s="72"/>
+      <c r="B80" s="77"/>
       <c r="C80" s="66"/>
       <c r="D80" s="67"/>
     </row>
@@ -14128,6 +14127,13 @@
     </row>
   </sheetData>
   <mergeCells count="19">
+    <mergeCell ref="A96:B96"/>
+    <mergeCell ref="A72:B72"/>
+    <mergeCell ref="A76:B76"/>
+    <mergeCell ref="A80:B80"/>
+    <mergeCell ref="A84:B84"/>
+    <mergeCell ref="A88:B88"/>
+    <mergeCell ref="A92:B92"/>
     <mergeCell ref="A68:B68"/>
     <mergeCell ref="A2:K2"/>
     <mergeCell ref="A3:A4"/>
@@ -14140,13 +14146,6 @@
     <mergeCell ref="A56:B56"/>
     <mergeCell ref="A60:B60"/>
     <mergeCell ref="A64:B64"/>
-    <mergeCell ref="A96:B96"/>
-    <mergeCell ref="A72:B72"/>
-    <mergeCell ref="A76:B76"/>
-    <mergeCell ref="A80:B80"/>
-    <mergeCell ref="A84:B84"/>
-    <mergeCell ref="A88:B88"/>
-    <mergeCell ref="A92:B92"/>
   </mergeCells>
   <pageMargins left="0.2" right="0.18" top="0.3" bottom="0.23" header="0.24" footer="0.23"/>
   <pageSetup paperSize="9" scale="70" orientation="portrait" horizontalDpi="4294967293" verticalDpi="1200" r:id="rId1"/>
@@ -14196,41 +14195,41 @@
       <c r="L1" s="2"/>
     </row>
     <row r="2" spans="1:16" ht="21" customHeight="1" thickBot="1">
-      <c r="A2" s="88" t="s">
+      <c r="A2" s="79" t="s">
         <v>64</v>
       </c>
-      <c r="B2" s="88"/>
-      <c r="C2" s="88"/>
-      <c r="D2" s="88"/>
-      <c r="E2" s="88"/>
-      <c r="F2" s="88"/>
-      <c r="G2" s="88"/>
-      <c r="H2" s="88"/>
-      <c r="I2" s="88"/>
-      <c r="J2" s="88"/>
-      <c r="K2" s="88"/>
+      <c r="B2" s="79"/>
+      <c r="C2" s="79"/>
+      <c r="D2" s="79"/>
+      <c r="E2" s="79"/>
+      <c r="F2" s="79"/>
+      <c r="G2" s="79"/>
+      <c r="H2" s="79"/>
+      <c r="I2" s="79"/>
+      <c r="J2" s="79"/>
+      <c r="K2" s="79"/>
       <c r="L2" s="2"/>
     </row>
     <row r="3" spans="1:16" s="6" customFormat="1" ht="21.6" customHeight="1" thickBot="1">
-      <c r="A3" s="89" t="s">
+      <c r="A3" s="80" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="90" t="s">
+      <c r="B3" s="81" t="s">
         <v>65</v>
       </c>
-      <c r="C3" s="90"/>
-      <c r="D3" s="90"/>
-      <c r="E3" s="90"/>
-      <c r="F3" s="90" t="s">
+      <c r="C3" s="81"/>
+      <c r="D3" s="81"/>
+      <c r="E3" s="81"/>
+      <c r="F3" s="81" t="s">
         <v>3</v>
       </c>
-      <c r="G3" s="90"/>
-      <c r="H3" s="90"/>
-      <c r="I3" s="90"/>
-      <c r="J3" s="90" t="s">
+      <c r="G3" s="81"/>
+      <c r="H3" s="81"/>
+      <c r="I3" s="81"/>
+      <c r="J3" s="81" t="s">
         <v>5</v>
       </c>
-      <c r="K3" s="90"/>
+      <c r="K3" s="81"/>
       <c r="M3" s="7" t="s">
         <v>6</v>
       </c>
@@ -14239,7 +14238,7 @@
       <c r="P3" s="8"/>
     </row>
     <row r="4" spans="1:16" s="6" customFormat="1" ht="54" customHeight="1" thickBot="1">
-      <c r="A4" s="89"/>
+      <c r="A4" s="80"/>
       <c r="B4" s="5" t="s">
         <v>7</v>
       </c>
@@ -15058,76 +15057,76 @@
     </row>
     <row r="40" spans="1:12" ht="21.95" customHeight="1"/>
     <row r="43" spans="1:12" ht="29.25" customHeight="1">
-      <c r="A43" s="91" t="s">
+      <c r="A43" s="82" t="s">
         <v>72</v>
       </c>
-      <c r="B43" s="92"/>
-      <c r="C43" s="92"/>
-      <c r="D43" s="92"/>
-      <c r="E43" s="92"/>
-      <c r="F43" s="92"/>
-      <c r="G43" s="92"/>
-      <c r="H43" s="92"/>
-      <c r="I43" s="92"/>
-      <c r="J43" s="92"/>
-      <c r="K43" s="92"/>
-      <c r="L43" s="92"/>
+      <c r="B43" s="83"/>
+      <c r="C43" s="83"/>
+      <c r="D43" s="83"/>
+      <c r="E43" s="83"/>
+      <c r="F43" s="83"/>
+      <c r="G43" s="83"/>
+      <c r="H43" s="83"/>
+      <c r="I43" s="83"/>
+      <c r="J43" s="83"/>
+      <c r="K43" s="83"/>
+      <c r="L43" s="83"/>
     </row>
     <row r="44" spans="1:12" ht="21.75" customHeight="1">
-      <c r="A44" s="92"/>
-      <c r="B44" s="92"/>
-      <c r="C44" s="92"/>
-      <c r="D44" s="92"/>
-      <c r="E44" s="92"/>
-      <c r="F44" s="92"/>
-      <c r="G44" s="92"/>
-      <c r="H44" s="92"/>
-      <c r="I44" s="92"/>
-      <c r="J44" s="92"/>
-      <c r="K44" s="92"/>
-      <c r="L44" s="92"/>
+      <c r="A44" s="83"/>
+      <c r="B44" s="83"/>
+      <c r="C44" s="83"/>
+      <c r="D44" s="83"/>
+      <c r="E44" s="83"/>
+      <c r="F44" s="83"/>
+      <c r="G44" s="83"/>
+      <c r="H44" s="83"/>
+      <c r="I44" s="83"/>
+      <c r="J44" s="83"/>
+      <c r="K44" s="83"/>
+      <c r="L44" s="83"/>
     </row>
     <row r="45" spans="1:12" ht="21.75" customHeight="1">
-      <c r="A45" s="92"/>
-      <c r="B45" s="92"/>
-      <c r="C45" s="92"/>
-      <c r="D45" s="92"/>
-      <c r="E45" s="92"/>
-      <c r="F45" s="92"/>
-      <c r="G45" s="92"/>
-      <c r="H45" s="92"/>
-      <c r="I45" s="92"/>
-      <c r="J45" s="92"/>
-      <c r="K45" s="92"/>
-      <c r="L45" s="92"/>
+      <c r="A45" s="83"/>
+      <c r="B45" s="83"/>
+      <c r="C45" s="83"/>
+      <c r="D45" s="83"/>
+      <c r="E45" s="83"/>
+      <c r="F45" s="83"/>
+      <c r="G45" s="83"/>
+      <c r="H45" s="83"/>
+      <c r="I45" s="83"/>
+      <c r="J45" s="83"/>
+      <c r="K45" s="83"/>
+      <c r="L45" s="83"/>
     </row>
     <row r="46" spans="1:12" ht="21.75" customHeight="1">
-      <c r="A46" s="92"/>
-      <c r="B46" s="92"/>
-      <c r="C46" s="92"/>
-      <c r="D46" s="92"/>
-      <c r="E46" s="92"/>
-      <c r="F46" s="92"/>
-      <c r="G46" s="92"/>
-      <c r="H46" s="92"/>
-      <c r="I46" s="92"/>
-      <c r="J46" s="92"/>
-      <c r="K46" s="92"/>
-      <c r="L46" s="92"/>
+      <c r="A46" s="83"/>
+      <c r="B46" s="83"/>
+      <c r="C46" s="83"/>
+      <c r="D46" s="83"/>
+      <c r="E46" s="83"/>
+      <c r="F46" s="83"/>
+      <c r="G46" s="83"/>
+      <c r="H46" s="83"/>
+      <c r="I46" s="83"/>
+      <c r="J46" s="83"/>
+      <c r="K46" s="83"/>
+      <c r="L46" s="83"/>
     </row>
     <row r="47" spans="1:12" ht="27" customHeight="1">
-      <c r="A47" s="92"/>
-      <c r="B47" s="92"/>
-      <c r="C47" s="92"/>
-      <c r="D47" s="92"/>
-      <c r="E47" s="92"/>
-      <c r="F47" s="92"/>
-      <c r="G47" s="92"/>
-      <c r="H47" s="92"/>
-      <c r="I47" s="92"/>
-      <c r="J47" s="92"/>
-      <c r="K47" s="92"/>
-      <c r="L47" s="92"/>
+      <c r="A47" s="83"/>
+      <c r="B47" s="83"/>
+      <c r="C47" s="83"/>
+      <c r="D47" s="83"/>
+      <c r="E47" s="83"/>
+      <c r="F47" s="83"/>
+      <c r="G47" s="83"/>
+      <c r="H47" s="83"/>
+      <c r="I47" s="83"/>
+      <c r="J47" s="83"/>
+      <c r="K47" s="83"/>
+      <c r="L47" s="83"/>
     </row>
     <row r="48" spans="1:12" ht="27" customHeight="1">
       <c r="A48" s="23"/>
@@ -15158,614 +15157,614 @@
       <c r="L49" s="23"/>
     </row>
     <row r="50" spans="1:12" ht="42" customHeight="1">
-      <c r="A50" s="77" t="s">
+      <c r="A50" s="76" t="s">
         <v>73</v>
       </c>
-      <c r="B50" s="77"/>
-      <c r="C50" s="77"/>
-      <c r="D50" s="77"/>
-      <c r="E50" s="77"/>
-      <c r="F50" s="77"/>
-      <c r="G50" s="77"/>
-      <c r="H50" s="77"/>
-      <c r="I50" s="77"/>
-      <c r="J50" s="77"/>
-      <c r="K50" s="77"/>
-      <c r="L50" s="77"/>
+      <c r="B50" s="76"/>
+      <c r="C50" s="76"/>
+      <c r="D50" s="76"/>
+      <c r="E50" s="76"/>
+      <c r="F50" s="76"/>
+      <c r="G50" s="76"/>
+      <c r="H50" s="76"/>
+      <c r="I50" s="76"/>
+      <c r="J50" s="76"/>
+      <c r="K50" s="76"/>
+      <c r="L50" s="76"/>
     </row>
     <row r="51" spans="1:12" s="24" customFormat="1" ht="30" customHeight="1">
-      <c r="A51" s="78" t="s">
+      <c r="A51" s="84" t="s">
         <v>74</v>
       </c>
-      <c r="B51" s="78"/>
-      <c r="C51" s="78"/>
-      <c r="D51" s="78"/>
-      <c r="E51" s="78"/>
-      <c r="F51" s="78"/>
-      <c r="G51" s="78"/>
-      <c r="H51" s="78"/>
-      <c r="I51" s="78"/>
-      <c r="J51" s="78"/>
-      <c r="K51" s="78"/>
-      <c r="L51" s="78"/>
+      <c r="B51" s="84"/>
+      <c r="C51" s="84"/>
+      <c r="D51" s="84"/>
+      <c r="E51" s="84"/>
+      <c r="F51" s="84"/>
+      <c r="G51" s="84"/>
+      <c r="H51" s="84"/>
+      <c r="I51" s="84"/>
+      <c r="J51" s="84"/>
+      <c r="K51" s="84"/>
+      <c r="L51" s="84"/>
     </row>
     <row r="52" spans="1:12" s="24" customFormat="1" ht="50.1" customHeight="1">
       <c r="A52" s="25" t="s">
         <v>49</v>
       </c>
-      <c r="B52" s="79" t="s">
+      <c r="B52" s="85" t="s">
         <v>75</v>
       </c>
-      <c r="C52" s="79"/>
-      <c r="D52" s="79"/>
-      <c r="E52" s="79"/>
-      <c r="F52" s="79"/>
-      <c r="G52" s="79"/>
-      <c r="H52" s="79"/>
-      <c r="I52" s="79"/>
-      <c r="J52" s="79"/>
-      <c r="K52" s="79"/>
-      <c r="L52" s="79"/>
+      <c r="C52" s="85"/>
+      <c r="D52" s="85"/>
+      <c r="E52" s="85"/>
+      <c r="F52" s="85"/>
+      <c r="G52" s="85"/>
+      <c r="H52" s="85"/>
+      <c r="I52" s="85"/>
+      <c r="J52" s="85"/>
+      <c r="K52" s="85"/>
+      <c r="L52" s="85"/>
     </row>
     <row r="53" spans="1:12" s="24" customFormat="1" ht="50.1" customHeight="1">
-      <c r="A53" s="83" t="s">
+      <c r="A53" s="86" t="s">
         <v>76</v>
       </c>
-      <c r="B53" s="83"/>
-      <c r="C53" s="81" t="s">
+      <c r="B53" s="86"/>
+      <c r="C53" s="78" t="s">
         <v>77</v>
       </c>
-      <c r="D53" s="81"/>
-      <c r="E53" s="81"/>
-      <c r="F53" s="81"/>
-      <c r="G53" s="81"/>
-      <c r="H53" s="81"/>
-      <c r="I53" s="81"/>
-      <c r="J53" s="81"/>
-      <c r="K53" s="81"/>
-      <c r="L53" s="81"/>
+      <c r="D53" s="78"/>
+      <c r="E53" s="78"/>
+      <c r="F53" s="78"/>
+      <c r="G53" s="78"/>
+      <c r="H53" s="78"/>
+      <c r="I53" s="78"/>
+      <c r="J53" s="78"/>
+      <c r="K53" s="78"/>
+      <c r="L53" s="78"/>
     </row>
     <row r="54" spans="1:12" s="24" customFormat="1" ht="50.1" customHeight="1">
       <c r="A54" s="25" t="s">
         <v>51</v>
       </c>
       <c r="B54" s="25"/>
-      <c r="C54" s="81" t="s">
+      <c r="C54" s="78" t="s">
         <v>78</v>
       </c>
-      <c r="D54" s="81"/>
-      <c r="E54" s="81"/>
-      <c r="F54" s="81"/>
-      <c r="G54" s="81"/>
-      <c r="H54" s="81"/>
-      <c r="I54" s="81"/>
-      <c r="J54" s="81"/>
-      <c r="K54" s="81"/>
-      <c r="L54" s="81"/>
+      <c r="D54" s="78"/>
+      <c r="E54" s="78"/>
+      <c r="F54" s="78"/>
+      <c r="G54" s="78"/>
+      <c r="H54" s="78"/>
+      <c r="I54" s="78"/>
+      <c r="J54" s="78"/>
+      <c r="K54" s="78"/>
+      <c r="L54" s="78"/>
     </row>
     <row r="55" spans="1:12" s="24" customFormat="1" ht="30" customHeight="1">
-      <c r="A55" s="78" t="s">
+      <c r="A55" s="84" t="s">
         <v>79</v>
       </c>
-      <c r="B55" s="78"/>
-      <c r="C55" s="78"/>
-      <c r="D55" s="78"/>
-      <c r="E55" s="78"/>
-      <c r="F55" s="78"/>
-      <c r="G55" s="78"/>
-      <c r="H55" s="78"/>
-      <c r="I55" s="78"/>
-      <c r="J55" s="78"/>
-      <c r="K55" s="78"/>
-      <c r="L55" s="78"/>
+      <c r="B55" s="84"/>
+      <c r="C55" s="84"/>
+      <c r="D55" s="84"/>
+      <c r="E55" s="84"/>
+      <c r="F55" s="84"/>
+      <c r="G55" s="84"/>
+      <c r="H55" s="84"/>
+      <c r="I55" s="84"/>
+      <c r="J55" s="84"/>
+      <c r="K55" s="84"/>
+      <c r="L55" s="84"/>
     </row>
     <row r="56" spans="1:12" s="24" customFormat="1" ht="50.1" customHeight="1">
       <c r="A56" s="25" t="s">
         <v>49</v>
       </c>
-      <c r="B56" s="79" t="s">
+      <c r="B56" s="85" t="s">
         <v>80</v>
       </c>
-      <c r="C56" s="79"/>
-      <c r="D56" s="79"/>
-      <c r="E56" s="79"/>
-      <c r="F56" s="79"/>
-      <c r="G56" s="79"/>
-      <c r="H56" s="79"/>
-      <c r="I56" s="79"/>
-      <c r="J56" s="79"/>
-      <c r="K56" s="79"/>
-      <c r="L56" s="79"/>
+      <c r="C56" s="85"/>
+      <c r="D56" s="85"/>
+      <c r="E56" s="85"/>
+      <c r="F56" s="85"/>
+      <c r="G56" s="85"/>
+      <c r="H56" s="85"/>
+      <c r="I56" s="85"/>
+      <c r="J56" s="85"/>
+      <c r="K56" s="85"/>
+      <c r="L56" s="85"/>
     </row>
     <row r="57" spans="1:12" s="24" customFormat="1" ht="50.1" customHeight="1">
-      <c r="A57" s="83" t="s">
+      <c r="A57" s="86" t="s">
         <v>76</v>
       </c>
-      <c r="B57" s="83"/>
-      <c r="C57" s="80" t="s">
+      <c r="B57" s="86"/>
+      <c r="C57" s="87" t="s">
         <v>81</v>
       </c>
-      <c r="D57" s="80"/>
-      <c r="E57" s="80"/>
-      <c r="F57" s="80"/>
-      <c r="G57" s="80"/>
-      <c r="H57" s="80"/>
-      <c r="I57" s="80"/>
-      <c r="J57" s="80"/>
-      <c r="K57" s="80"/>
-      <c r="L57" s="80"/>
+      <c r="D57" s="87"/>
+      <c r="E57" s="87"/>
+      <c r="F57" s="87"/>
+      <c r="G57" s="87"/>
+      <c r="H57" s="87"/>
+      <c r="I57" s="87"/>
+      <c r="J57" s="87"/>
+      <c r="K57" s="87"/>
+      <c r="L57" s="87"/>
     </row>
     <row r="58" spans="1:12" s="24" customFormat="1" ht="50.1" customHeight="1">
       <c r="A58" s="25" t="s">
         <v>51</v>
       </c>
-      <c r="B58" s="87" t="s">
+      <c r="B58" s="88" t="s">
         <v>78</v>
       </c>
-      <c r="C58" s="81"/>
-      <c r="D58" s="81"/>
-      <c r="E58" s="81"/>
-      <c r="F58" s="81"/>
-      <c r="G58" s="81"/>
-      <c r="H58" s="81"/>
-      <c r="I58" s="81"/>
-      <c r="J58" s="81"/>
-      <c r="K58" s="81"/>
-      <c r="L58" s="81"/>
+      <c r="C58" s="78"/>
+      <c r="D58" s="78"/>
+      <c r="E58" s="78"/>
+      <c r="F58" s="78"/>
+      <c r="G58" s="78"/>
+      <c r="H58" s="78"/>
+      <c r="I58" s="78"/>
+      <c r="J58" s="78"/>
+      <c r="K58" s="78"/>
+      <c r="L58" s="78"/>
     </row>
     <row r="59" spans="1:12" s="24" customFormat="1" ht="30" customHeight="1">
-      <c r="A59" s="78" t="s">
+      <c r="A59" s="84" t="s">
         <v>82</v>
       </c>
-      <c r="B59" s="78"/>
-      <c r="C59" s="78"/>
-      <c r="D59" s="78"/>
-      <c r="E59" s="78"/>
-      <c r="F59" s="78"/>
-      <c r="G59" s="78"/>
-      <c r="H59" s="78"/>
-      <c r="I59" s="78"/>
-      <c r="J59" s="78"/>
-      <c r="K59" s="78"/>
-      <c r="L59" s="78"/>
+      <c r="B59" s="84"/>
+      <c r="C59" s="84"/>
+      <c r="D59" s="84"/>
+      <c r="E59" s="84"/>
+      <c r="F59" s="84"/>
+      <c r="G59" s="84"/>
+      <c r="H59" s="84"/>
+      <c r="I59" s="84"/>
+      <c r="J59" s="84"/>
+      <c r="K59" s="84"/>
+      <c r="L59" s="84"/>
     </row>
     <row r="60" spans="1:12" s="24" customFormat="1" ht="50.1" customHeight="1">
       <c r="A60" s="25" t="s">
         <v>49</v>
       </c>
-      <c r="B60" s="79" t="s">
+      <c r="B60" s="85" t="s">
         <v>83</v>
       </c>
-      <c r="C60" s="79"/>
-      <c r="D60" s="79"/>
-      <c r="E60" s="79"/>
-      <c r="F60" s="79"/>
-      <c r="G60" s="79"/>
-      <c r="H60" s="79"/>
-      <c r="I60" s="79"/>
-      <c r="J60" s="79"/>
-      <c r="K60" s="79"/>
-      <c r="L60" s="79"/>
+      <c r="C60" s="85"/>
+      <c r="D60" s="85"/>
+      <c r="E60" s="85"/>
+      <c r="F60" s="85"/>
+      <c r="G60" s="85"/>
+      <c r="H60" s="85"/>
+      <c r="I60" s="85"/>
+      <c r="J60" s="85"/>
+      <c r="K60" s="85"/>
+      <c r="L60" s="85"/>
     </row>
     <row r="61" spans="1:12" s="24" customFormat="1" ht="50.1" customHeight="1">
-      <c r="A61" s="83" t="s">
+      <c r="A61" s="86" t="s">
         <v>76</v>
       </c>
-      <c r="B61" s="83"/>
-      <c r="C61" s="80" t="s">
+      <c r="B61" s="86"/>
+      <c r="C61" s="87" t="s">
         <v>84</v>
       </c>
-      <c r="D61" s="80"/>
-      <c r="E61" s="80"/>
-      <c r="F61" s="80"/>
-      <c r="G61" s="80"/>
-      <c r="H61" s="80"/>
-      <c r="I61" s="80"/>
-      <c r="J61" s="80"/>
-      <c r="K61" s="80"/>
-      <c r="L61" s="80"/>
+      <c r="D61" s="87"/>
+      <c r="E61" s="87"/>
+      <c r="F61" s="87"/>
+      <c r="G61" s="87"/>
+      <c r="H61" s="87"/>
+      <c r="I61" s="87"/>
+      <c r="J61" s="87"/>
+      <c r="K61" s="87"/>
+      <c r="L61" s="87"/>
     </row>
     <row r="62" spans="1:12" s="24" customFormat="1" ht="50.1" customHeight="1">
       <c r="A62" s="25" t="s">
         <v>51</v>
       </c>
       <c r="B62" s="25"/>
-      <c r="C62" s="80" t="s">
+      <c r="C62" s="87" t="s">
         <v>85</v>
       </c>
-      <c r="D62" s="80"/>
-      <c r="E62" s="80"/>
-      <c r="F62" s="80"/>
-      <c r="G62" s="80"/>
-      <c r="H62" s="80"/>
-      <c r="I62" s="80"/>
-      <c r="J62" s="80"/>
-      <c r="K62" s="80"/>
-      <c r="L62" s="80"/>
+      <c r="D62" s="87"/>
+      <c r="E62" s="87"/>
+      <c r="F62" s="87"/>
+      <c r="G62" s="87"/>
+      <c r="H62" s="87"/>
+      <c r="I62" s="87"/>
+      <c r="J62" s="87"/>
+      <c r="K62" s="87"/>
+      <c r="L62" s="87"/>
     </row>
     <row r="63" spans="1:12" s="24" customFormat="1" ht="30" customHeight="1">
-      <c r="A63" s="78" t="s">
+      <c r="A63" s="84" t="s">
         <v>86</v>
       </c>
-      <c r="B63" s="78"/>
-      <c r="C63" s="78"/>
-      <c r="D63" s="78"/>
-      <c r="E63" s="78"/>
-      <c r="F63" s="78"/>
-      <c r="G63" s="78"/>
-      <c r="H63" s="78"/>
-      <c r="I63" s="78"/>
-      <c r="J63" s="78"/>
-      <c r="K63" s="78"/>
-      <c r="L63" s="78"/>
+      <c r="B63" s="84"/>
+      <c r="C63" s="84"/>
+      <c r="D63" s="84"/>
+      <c r="E63" s="84"/>
+      <c r="F63" s="84"/>
+      <c r="G63" s="84"/>
+      <c r="H63" s="84"/>
+      <c r="I63" s="84"/>
+      <c r="J63" s="84"/>
+      <c r="K63" s="84"/>
+      <c r="L63" s="84"/>
     </row>
     <row r="64" spans="1:12" s="24" customFormat="1" ht="50.1" customHeight="1">
       <c r="A64" s="26" t="s">
         <v>87</v>
       </c>
       <c r="B64" s="25"/>
-      <c r="C64" s="79" t="s">
+      <c r="C64" s="85" t="s">
         <v>88</v>
       </c>
-      <c r="D64" s="79"/>
-      <c r="E64" s="79"/>
-      <c r="F64" s="79"/>
-      <c r="G64" s="79"/>
-      <c r="H64" s="79"/>
-      <c r="I64" s="79"/>
-      <c r="J64" s="79"/>
-      <c r="K64" s="79"/>
-      <c r="L64" s="79"/>
+      <c r="D64" s="85"/>
+      <c r="E64" s="85"/>
+      <c r="F64" s="85"/>
+      <c r="G64" s="85"/>
+      <c r="H64" s="85"/>
+      <c r="I64" s="85"/>
+      <c r="J64" s="85"/>
+      <c r="K64" s="85"/>
+      <c r="L64" s="85"/>
     </row>
     <row r="65" spans="1:12" s="24" customFormat="1" ht="50.1" customHeight="1">
-      <c r="A65" s="79" t="s">
+      <c r="A65" s="85" t="s">
         <v>50</v>
       </c>
-      <c r="B65" s="79"/>
-      <c r="C65" s="80" t="s">
+      <c r="B65" s="85"/>
+      <c r="C65" s="87" t="s">
         <v>89</v>
       </c>
-      <c r="D65" s="80"/>
-      <c r="E65" s="80"/>
-      <c r="F65" s="80"/>
-      <c r="G65" s="80"/>
-      <c r="H65" s="80"/>
-      <c r="I65" s="80"/>
-      <c r="J65" s="80"/>
-      <c r="K65" s="80"/>
-      <c r="L65" s="80"/>
+      <c r="D65" s="87"/>
+      <c r="E65" s="87"/>
+      <c r="F65" s="87"/>
+      <c r="G65" s="87"/>
+      <c r="H65" s="87"/>
+      <c r="I65" s="87"/>
+      <c r="J65" s="87"/>
+      <c r="K65" s="87"/>
+      <c r="L65" s="87"/>
     </row>
     <row r="66" spans="1:12" s="24" customFormat="1" ht="50.1" customHeight="1">
       <c r="A66" s="25" t="s">
         <v>51</v>
       </c>
       <c r="B66" s="25"/>
-      <c r="C66" s="81" t="s">
+      <c r="C66" s="78" t="s">
         <v>90</v>
       </c>
-      <c r="D66" s="81"/>
-      <c r="E66" s="81"/>
-      <c r="F66" s="81"/>
-      <c r="G66" s="81"/>
-      <c r="H66" s="81"/>
-      <c r="I66" s="81"/>
-      <c r="J66" s="81"/>
-      <c r="K66" s="81"/>
-      <c r="L66" s="81"/>
+      <c r="D66" s="78"/>
+      <c r="E66" s="78"/>
+      <c r="F66" s="78"/>
+      <c r="G66" s="78"/>
+      <c r="H66" s="78"/>
+      <c r="I66" s="78"/>
+      <c r="J66" s="78"/>
+      <c r="K66" s="78"/>
+      <c r="L66" s="78"/>
     </row>
     <row r="67" spans="1:12" s="24" customFormat="1" ht="30" customHeight="1">
-      <c r="A67" s="78" t="s">
+      <c r="A67" s="84" t="s">
         <v>91</v>
       </c>
-      <c r="B67" s="78"/>
-      <c r="C67" s="78"/>
-      <c r="D67" s="78"/>
-      <c r="E67" s="78"/>
-      <c r="F67" s="78"/>
-      <c r="G67" s="78"/>
-      <c r="H67" s="78"/>
-      <c r="I67" s="78"/>
-      <c r="J67" s="78"/>
-      <c r="K67" s="78"/>
-      <c r="L67" s="78"/>
+      <c r="B67" s="84"/>
+      <c r="C67" s="84"/>
+      <c r="D67" s="84"/>
+      <c r="E67" s="84"/>
+      <c r="F67" s="84"/>
+      <c r="G67" s="84"/>
+      <c r="H67" s="84"/>
+      <c r="I67" s="84"/>
+      <c r="J67" s="84"/>
+      <c r="K67" s="84"/>
+      <c r="L67" s="84"/>
     </row>
     <row r="68" spans="1:12" s="24" customFormat="1" ht="50.1" customHeight="1">
       <c r="A68" s="26" t="s">
         <v>87</v>
       </c>
       <c r="B68" s="25"/>
-      <c r="C68" s="79" t="s">
+      <c r="C68" s="85" t="s">
         <v>92</v>
       </c>
-      <c r="D68" s="79"/>
-      <c r="E68" s="79"/>
-      <c r="F68" s="79"/>
-      <c r="G68" s="79"/>
-      <c r="H68" s="79"/>
-      <c r="I68" s="79"/>
-      <c r="J68" s="79"/>
-      <c r="K68" s="79"/>
-      <c r="L68" s="79"/>
+      <c r="D68" s="85"/>
+      <c r="E68" s="85"/>
+      <c r="F68" s="85"/>
+      <c r="G68" s="85"/>
+      <c r="H68" s="85"/>
+      <c r="I68" s="85"/>
+      <c r="J68" s="85"/>
+      <c r="K68" s="85"/>
+      <c r="L68" s="85"/>
     </row>
     <row r="69" spans="1:12" s="24" customFormat="1" ht="50.1" customHeight="1">
-      <c r="A69" s="79" t="s">
+      <c r="A69" s="85" t="s">
         <v>50</v>
       </c>
-      <c r="B69" s="79"/>
-      <c r="C69" s="80" t="s">
+      <c r="B69" s="85"/>
+      <c r="C69" s="87" t="s">
         <v>93</v>
       </c>
-      <c r="D69" s="80"/>
-      <c r="E69" s="80"/>
-      <c r="F69" s="80"/>
-      <c r="G69" s="80"/>
-      <c r="H69" s="80"/>
-      <c r="I69" s="80"/>
-      <c r="J69" s="80"/>
-      <c r="K69" s="80"/>
-      <c r="L69" s="80"/>
+      <c r="D69" s="87"/>
+      <c r="E69" s="87"/>
+      <c r="F69" s="87"/>
+      <c r="G69" s="87"/>
+      <c r="H69" s="87"/>
+      <c r="I69" s="87"/>
+      <c r="J69" s="87"/>
+      <c r="K69" s="87"/>
+      <c r="L69" s="87"/>
     </row>
     <row r="70" spans="1:12" s="24" customFormat="1" ht="50.1" customHeight="1">
       <c r="A70" s="25" t="s">
         <v>51</v>
       </c>
       <c r="B70" s="25"/>
-      <c r="C70" s="84" t="s">
+      <c r="C70" s="89" t="s">
         <v>94</v>
       </c>
-      <c r="D70" s="84"/>
-      <c r="E70" s="84"/>
-      <c r="F70" s="84"/>
-      <c r="G70" s="84"/>
-      <c r="H70" s="84"/>
-      <c r="I70" s="84"/>
-      <c r="J70" s="84"/>
-      <c r="K70" s="84"/>
-      <c r="L70" s="84"/>
+      <c r="D70" s="89"/>
+      <c r="E70" s="89"/>
+      <c r="F70" s="89"/>
+      <c r="G70" s="89"/>
+      <c r="H70" s="89"/>
+      <c r="I70" s="89"/>
+      <c r="J70" s="89"/>
+      <c r="K70" s="89"/>
+      <c r="L70" s="89"/>
     </row>
     <row r="71" spans="1:12" s="24" customFormat="1" ht="30" customHeight="1">
-      <c r="A71" s="78" t="s">
+      <c r="A71" s="84" t="s">
         <v>95</v>
       </c>
-      <c r="B71" s="78"/>
-      <c r="C71" s="78"/>
-      <c r="D71" s="78"/>
-      <c r="E71" s="78"/>
-      <c r="F71" s="78"/>
-      <c r="G71" s="78"/>
-      <c r="H71" s="78"/>
-      <c r="I71" s="78"/>
-      <c r="J71" s="78"/>
-      <c r="K71" s="78"/>
-      <c r="L71" s="78"/>
+      <c r="B71" s="84"/>
+      <c r="C71" s="84"/>
+      <c r="D71" s="84"/>
+      <c r="E71" s="84"/>
+      <c r="F71" s="84"/>
+      <c r="G71" s="84"/>
+      <c r="H71" s="84"/>
+      <c r="I71" s="84"/>
+      <c r="J71" s="84"/>
+      <c r="K71" s="84"/>
+      <c r="L71" s="84"/>
     </row>
     <row r="72" spans="1:12" s="24" customFormat="1" ht="50.1" customHeight="1">
       <c r="A72" s="26" t="s">
         <v>87</v>
       </c>
       <c r="B72" s="25"/>
-      <c r="C72" s="79" t="s">
+      <c r="C72" s="85" t="s">
         <v>96</v>
       </c>
-      <c r="D72" s="79"/>
-      <c r="E72" s="79"/>
-      <c r="F72" s="79"/>
-      <c r="G72" s="79"/>
-      <c r="H72" s="79"/>
-      <c r="I72" s="79"/>
-      <c r="J72" s="79"/>
-      <c r="K72" s="79"/>
-      <c r="L72" s="79"/>
+      <c r="D72" s="85"/>
+      <c r="E72" s="85"/>
+      <c r="F72" s="85"/>
+      <c r="G72" s="85"/>
+      <c r="H72" s="85"/>
+      <c r="I72" s="85"/>
+      <c r="J72" s="85"/>
+      <c r="K72" s="85"/>
+      <c r="L72" s="85"/>
     </row>
     <row r="73" spans="1:12" s="24" customFormat="1" ht="50.1" customHeight="1">
-      <c r="A73" s="79" t="s">
+      <c r="A73" s="85" t="s">
         <v>50</v>
       </c>
-      <c r="B73" s="79"/>
-      <c r="C73" s="85" t="s">
+      <c r="B73" s="85"/>
+      <c r="C73" s="90" t="s">
         <v>97</v>
       </c>
-      <c r="D73" s="86"/>
-      <c r="E73" s="86"/>
-      <c r="F73" s="86"/>
-      <c r="G73" s="86"/>
-      <c r="H73" s="86"/>
-      <c r="I73" s="86"/>
-      <c r="J73" s="86"/>
-      <c r="K73" s="86"/>
-      <c r="L73" s="86"/>
+      <c r="D73" s="91"/>
+      <c r="E73" s="91"/>
+      <c r="F73" s="91"/>
+      <c r="G73" s="91"/>
+      <c r="H73" s="91"/>
+      <c r="I73" s="91"/>
+      <c r="J73" s="91"/>
+      <c r="K73" s="91"/>
+      <c r="L73" s="91"/>
     </row>
     <row r="74" spans="1:12" s="24" customFormat="1" ht="50.1" customHeight="1">
       <c r="A74" s="25" t="s">
         <v>51</v>
       </c>
       <c r="B74" s="25"/>
-      <c r="C74" s="81" t="s">
+      <c r="C74" s="78" t="s">
         <v>98</v>
       </c>
-      <c r="D74" s="81"/>
-      <c r="E74" s="81"/>
-      <c r="F74" s="81"/>
-      <c r="G74" s="81"/>
-      <c r="H74" s="81"/>
-      <c r="I74" s="81"/>
-      <c r="J74" s="81"/>
-      <c r="K74" s="81"/>
-      <c r="L74" s="81"/>
+      <c r="D74" s="78"/>
+      <c r="E74" s="78"/>
+      <c r="F74" s="78"/>
+      <c r="G74" s="78"/>
+      <c r="H74" s="78"/>
+      <c r="I74" s="78"/>
+      <c r="J74" s="78"/>
+      <c r="K74" s="78"/>
+      <c r="L74" s="78"/>
     </row>
     <row r="75" spans="1:12" s="24" customFormat="1" ht="30" customHeight="1">
-      <c r="A75" s="78" t="s">
+      <c r="A75" s="84" t="s">
         <v>99</v>
       </c>
-      <c r="B75" s="78"/>
-      <c r="C75" s="78"/>
-      <c r="D75" s="78"/>
-      <c r="E75" s="78"/>
-      <c r="F75" s="78"/>
-      <c r="G75" s="78"/>
-      <c r="H75" s="78"/>
-      <c r="I75" s="78"/>
-      <c r="J75" s="78"/>
-      <c r="K75" s="78"/>
-      <c r="L75" s="78"/>
+      <c r="B75" s="84"/>
+      <c r="C75" s="84"/>
+      <c r="D75" s="84"/>
+      <c r="E75" s="84"/>
+      <c r="F75" s="84"/>
+      <c r="G75" s="84"/>
+      <c r="H75" s="84"/>
+      <c r="I75" s="84"/>
+      <c r="J75" s="84"/>
+      <c r="K75" s="84"/>
+      <c r="L75" s="84"/>
     </row>
     <row r="76" spans="1:12" s="24" customFormat="1" ht="39.950000000000003" customHeight="1">
       <c r="A76" s="25" t="s">
         <v>49</v>
       </c>
       <c r="B76" s="25"/>
-      <c r="C76" s="79" t="s">
+      <c r="C76" s="85" t="s">
         <v>100</v>
       </c>
-      <c r="D76" s="79"/>
-      <c r="E76" s="79"/>
-      <c r="F76" s="79"/>
-      <c r="G76" s="79"/>
-      <c r="H76" s="79"/>
-      <c r="I76" s="79"/>
-      <c r="J76" s="79"/>
-      <c r="K76" s="79"/>
-      <c r="L76" s="79"/>
+      <c r="D76" s="85"/>
+      <c r="E76" s="85"/>
+      <c r="F76" s="85"/>
+      <c r="G76" s="85"/>
+      <c r="H76" s="85"/>
+      <c r="I76" s="85"/>
+      <c r="J76" s="85"/>
+      <c r="K76" s="85"/>
+      <c r="L76" s="85"/>
     </row>
     <row r="77" spans="1:12" s="24" customFormat="1" ht="39.950000000000003" customHeight="1">
-      <c r="A77" s="83" t="s">
+      <c r="A77" s="86" t="s">
         <v>50</v>
       </c>
-      <c r="B77" s="83"/>
-      <c r="C77" s="80" t="s">
+      <c r="B77" s="86"/>
+      <c r="C77" s="87" t="s">
         <v>101</v>
       </c>
-      <c r="D77" s="80"/>
-      <c r="E77" s="80"/>
-      <c r="F77" s="80"/>
-      <c r="G77" s="80"/>
-      <c r="H77" s="80"/>
-      <c r="I77" s="80"/>
-      <c r="J77" s="80"/>
-      <c r="K77" s="80"/>
-      <c r="L77" s="80"/>
+      <c r="D77" s="87"/>
+      <c r="E77" s="87"/>
+      <c r="F77" s="87"/>
+      <c r="G77" s="87"/>
+      <c r="H77" s="87"/>
+      <c r="I77" s="87"/>
+      <c r="J77" s="87"/>
+      <c r="K77" s="87"/>
+      <c r="L77" s="87"/>
     </row>
     <row r="78" spans="1:12" s="24" customFormat="1" ht="39.950000000000003" customHeight="1">
       <c r="A78" s="25" t="s">
         <v>51</v>
       </c>
       <c r="B78" s="25"/>
-      <c r="C78" s="81" t="s">
+      <c r="C78" s="78" t="s">
         <v>78</v>
       </c>
-      <c r="D78" s="81"/>
-      <c r="E78" s="81"/>
-      <c r="F78" s="81"/>
-      <c r="G78" s="81"/>
-      <c r="H78" s="81"/>
-      <c r="I78" s="81"/>
-      <c r="J78" s="81"/>
-      <c r="K78" s="81"/>
-      <c r="L78" s="81"/>
+      <c r="D78" s="78"/>
+      <c r="E78" s="78"/>
+      <c r="F78" s="78"/>
+      <c r="G78" s="78"/>
+      <c r="H78" s="78"/>
+      <c r="I78" s="78"/>
+      <c r="J78" s="78"/>
+      <c r="K78" s="78"/>
+      <c r="L78" s="78"/>
     </row>
     <row r="79" spans="1:12" s="24" customFormat="1" ht="30" customHeight="1">
-      <c r="A79" s="78" t="s">
+      <c r="A79" s="84" t="s">
         <v>102</v>
       </c>
-      <c r="B79" s="78"/>
-      <c r="C79" s="78"/>
-      <c r="D79" s="78"/>
-      <c r="E79" s="78"/>
-      <c r="F79" s="78"/>
-      <c r="G79" s="78"/>
-      <c r="H79" s="78"/>
-      <c r="I79" s="78"/>
-      <c r="J79" s="78"/>
-      <c r="K79" s="78"/>
-      <c r="L79" s="78"/>
+      <c r="B79" s="84"/>
+      <c r="C79" s="84"/>
+      <c r="D79" s="84"/>
+      <c r="E79" s="84"/>
+      <c r="F79" s="84"/>
+      <c r="G79" s="84"/>
+      <c r="H79" s="84"/>
+      <c r="I79" s="84"/>
+      <c r="J79" s="84"/>
+      <c r="K79" s="84"/>
+      <c r="L79" s="84"/>
     </row>
     <row r="80" spans="1:12" s="24" customFormat="1" ht="39.950000000000003" customHeight="1">
       <c r="A80" s="25" t="s">
         <v>49</v>
       </c>
       <c r="B80" s="25"/>
-      <c r="C80" s="79" t="s">
+      <c r="C80" s="85" t="s">
         <v>103</v>
       </c>
-      <c r="D80" s="79"/>
-      <c r="E80" s="79"/>
-      <c r="F80" s="79"/>
-      <c r="G80" s="79"/>
-      <c r="H80" s="79"/>
-      <c r="I80" s="79"/>
-      <c r="J80" s="79"/>
-      <c r="K80" s="79"/>
-      <c r="L80" s="79"/>
+      <c r="D80" s="85"/>
+      <c r="E80" s="85"/>
+      <c r="F80" s="85"/>
+      <c r="G80" s="85"/>
+      <c r="H80" s="85"/>
+      <c r="I80" s="85"/>
+      <c r="J80" s="85"/>
+      <c r="K80" s="85"/>
+      <c r="L80" s="85"/>
     </row>
     <row r="81" spans="1:20" s="24" customFormat="1" ht="39.950000000000003" customHeight="1">
-      <c r="A81" s="83" t="s">
+      <c r="A81" s="86" t="s">
         <v>50</v>
       </c>
-      <c r="B81" s="83"/>
-      <c r="C81" s="80" t="s">
+      <c r="B81" s="86"/>
+      <c r="C81" s="87" t="s">
         <v>104</v>
       </c>
-      <c r="D81" s="80"/>
-      <c r="E81" s="80"/>
-      <c r="F81" s="80"/>
-      <c r="G81" s="80"/>
-      <c r="H81" s="80"/>
-      <c r="I81" s="80"/>
-      <c r="J81" s="80"/>
-      <c r="K81" s="80"/>
-      <c r="L81" s="80"/>
+      <c r="D81" s="87"/>
+      <c r="E81" s="87"/>
+      <c r="F81" s="87"/>
+      <c r="G81" s="87"/>
+      <c r="H81" s="87"/>
+      <c r="I81" s="87"/>
+      <c r="J81" s="87"/>
+      <c r="K81" s="87"/>
+      <c r="L81" s="87"/>
     </row>
     <row r="82" spans="1:20" s="24" customFormat="1" ht="39.950000000000003" customHeight="1">
       <c r="A82" s="25" t="s">
         <v>51</v>
       </c>
       <c r="B82" s="25"/>
-      <c r="C82" s="81" t="s">
+      <c r="C82" s="78" t="s">
         <v>78</v>
       </c>
-      <c r="D82" s="81"/>
-      <c r="E82" s="81"/>
-      <c r="F82" s="81"/>
-      <c r="G82" s="81"/>
-      <c r="H82" s="81"/>
-      <c r="I82" s="81"/>
-      <c r="J82" s="81"/>
-      <c r="K82" s="81"/>
-      <c r="L82" s="81"/>
+      <c r="D82" s="78"/>
+      <c r="E82" s="78"/>
+      <c r="F82" s="78"/>
+      <c r="G82" s="78"/>
+      <c r="H82" s="78"/>
+      <c r="I82" s="78"/>
+      <c r="J82" s="78"/>
+      <c r="K82" s="78"/>
+      <c r="L82" s="78"/>
     </row>
     <row r="83" spans="1:20" s="24" customFormat="1" ht="30" customHeight="1">
-      <c r="A83" s="78" t="s">
+      <c r="A83" s="84" t="s">
         <v>105</v>
       </c>
-      <c r="B83" s="78"/>
-      <c r="C83" s="78"/>
-      <c r="D83" s="78"/>
-      <c r="E83" s="78"/>
-      <c r="F83" s="78"/>
-      <c r="G83" s="78"/>
-      <c r="H83" s="78"/>
-      <c r="I83" s="78"/>
-      <c r="J83" s="78"/>
-      <c r="K83" s="78"/>
-      <c r="L83" s="78"/>
+      <c r="B83" s="84"/>
+      <c r="C83" s="84"/>
+      <c r="D83" s="84"/>
+      <c r="E83" s="84"/>
+      <c r="F83" s="84"/>
+      <c r="G83" s="84"/>
+      <c r="H83" s="84"/>
+      <c r="I83" s="84"/>
+      <c r="J83" s="84"/>
+      <c r="K83" s="84"/>
+      <c r="L83" s="84"/>
     </row>
     <row r="84" spans="1:20" s="24" customFormat="1" ht="39.950000000000003" customHeight="1">
       <c r="A84" s="25" t="s">
         <v>49</v>
       </c>
       <c r="B84" s="25"/>
-      <c r="C84" s="79" t="s">
+      <c r="C84" s="85" t="s">
         <v>106</v>
       </c>
-      <c r="D84" s="79"/>
-      <c r="E84" s="79"/>
-      <c r="F84" s="79"/>
-      <c r="G84" s="79"/>
-      <c r="H84" s="79"/>
-      <c r="I84" s="79"/>
-      <c r="J84" s="79"/>
-      <c r="K84" s="79"/>
-      <c r="L84" s="79"/>
+      <c r="D84" s="85"/>
+      <c r="E84" s="85"/>
+      <c r="F84" s="85"/>
+      <c r="G84" s="85"/>
+      <c r="H84" s="85"/>
+      <c r="I84" s="85"/>
+      <c r="J84" s="85"/>
+      <c r="K84" s="85"/>
+      <c r="L84" s="85"/>
       <c r="M84" s="27"/>
       <c r="N84" s="27"/>
       <c r="O84" s="27"/>
@@ -15776,22 +15775,22 @@
       <c r="T84" s="27"/>
     </row>
     <row r="85" spans="1:20" s="24" customFormat="1" ht="39.950000000000003" customHeight="1">
-      <c r="A85" s="79" t="s">
+      <c r="A85" s="85" t="s">
         <v>50</v>
       </c>
-      <c r="B85" s="79"/>
-      <c r="C85" s="80" t="s">
+      <c r="B85" s="85"/>
+      <c r="C85" s="87" t="s">
         <v>107</v>
       </c>
-      <c r="D85" s="80"/>
-      <c r="E85" s="80"/>
-      <c r="F85" s="80"/>
-      <c r="G85" s="80"/>
-      <c r="H85" s="80"/>
-      <c r="I85" s="80"/>
-      <c r="J85" s="80"/>
-      <c r="K85" s="80"/>
-      <c r="L85" s="80"/>
+      <c r="D85" s="87"/>
+      <c r="E85" s="87"/>
+      <c r="F85" s="87"/>
+      <c r="G85" s="87"/>
+      <c r="H85" s="87"/>
+      <c r="I85" s="87"/>
+      <c r="J85" s="87"/>
+      <c r="K85" s="87"/>
+      <c r="L85" s="87"/>
       <c r="M85" s="27"/>
       <c r="N85" s="27"/>
       <c r="O85" s="27"/>
@@ -15806,18 +15805,18 @@
         <v>51</v>
       </c>
       <c r="B86" s="25"/>
-      <c r="C86" s="81" t="s">
+      <c r="C86" s="78" t="s">
         <v>78</v>
       </c>
-      <c r="D86" s="81"/>
-      <c r="E86" s="81"/>
-      <c r="F86" s="81"/>
-      <c r="G86" s="81"/>
-      <c r="H86" s="81"/>
-      <c r="I86" s="81"/>
-      <c r="J86" s="81"/>
-      <c r="K86" s="81"/>
-      <c r="L86" s="81"/>
+      <c r="D86" s="78"/>
+      <c r="E86" s="78"/>
+      <c r="F86" s="78"/>
+      <c r="G86" s="78"/>
+      <c r="H86" s="78"/>
+      <c r="I86" s="78"/>
+      <c r="J86" s="78"/>
+      <c r="K86" s="78"/>
+      <c r="L86" s="78"/>
       <c r="M86" s="27"/>
       <c r="N86" s="27"/>
       <c r="O86" s="27"/>
@@ -15828,214 +15827,214 @@
       <c r="T86" s="27"/>
     </row>
     <row r="87" spans="1:20" s="24" customFormat="1" ht="30" customHeight="1">
-      <c r="A87" s="78" t="s">
+      <c r="A87" s="84" t="s">
         <v>108</v>
       </c>
-      <c r="B87" s="78"/>
-      <c r="C87" s="78"/>
-      <c r="D87" s="78"/>
-      <c r="E87" s="78"/>
-      <c r="F87" s="78"/>
-      <c r="G87" s="78"/>
-      <c r="H87" s="78"/>
-      <c r="I87" s="78"/>
-      <c r="J87" s="78"/>
-      <c r="K87" s="78"/>
-      <c r="L87" s="78"/>
+      <c r="B87" s="84"/>
+      <c r="C87" s="84"/>
+      <c r="D87" s="84"/>
+      <c r="E87" s="84"/>
+      <c r="F87" s="84"/>
+      <c r="G87" s="84"/>
+      <c r="H87" s="84"/>
+      <c r="I87" s="84"/>
+      <c r="J87" s="84"/>
+      <c r="K87" s="84"/>
+      <c r="L87" s="84"/>
     </row>
     <row r="88" spans="1:20" s="28" customFormat="1" ht="39.950000000000003" customHeight="1">
       <c r="A88" s="25" t="s">
         <v>49</v>
       </c>
       <c r="B88" s="25"/>
-      <c r="C88" s="79" t="s">
+      <c r="C88" s="85" t="s">
         <v>109</v>
       </c>
-      <c r="D88" s="79"/>
-      <c r="E88" s="79"/>
-      <c r="F88" s="79"/>
-      <c r="G88" s="79"/>
-      <c r="H88" s="79"/>
-      <c r="I88" s="79"/>
-      <c r="J88" s="79"/>
-      <c r="K88" s="79"/>
-      <c r="L88" s="79"/>
+      <c r="D88" s="85"/>
+      <c r="E88" s="85"/>
+      <c r="F88" s="85"/>
+      <c r="G88" s="85"/>
+      <c r="H88" s="85"/>
+      <c r="I88" s="85"/>
+      <c r="J88" s="85"/>
+      <c r="K88" s="85"/>
+      <c r="L88" s="85"/>
     </row>
     <row r="89" spans="1:20" s="28" customFormat="1" ht="39.950000000000003" customHeight="1">
-      <c r="A89" s="79" t="s">
+      <c r="A89" s="85" t="s">
         <v>50</v>
       </c>
-      <c r="B89" s="79"/>
-      <c r="C89" s="82" t="s">
+      <c r="B89" s="85"/>
+      <c r="C89" s="92" t="s">
         <v>110</v>
       </c>
-      <c r="D89" s="79"/>
-      <c r="E89" s="79"/>
-      <c r="F89" s="79"/>
-      <c r="G89" s="79"/>
-      <c r="H89" s="79"/>
-      <c r="I89" s="79"/>
-      <c r="J89" s="79"/>
-      <c r="K89" s="79"/>
-      <c r="L89" s="79"/>
+      <c r="D89" s="85"/>
+      <c r="E89" s="85"/>
+      <c r="F89" s="85"/>
+      <c r="G89" s="85"/>
+      <c r="H89" s="85"/>
+      <c r="I89" s="85"/>
+      <c r="J89" s="85"/>
+      <c r="K89" s="85"/>
+      <c r="L89" s="85"/>
     </row>
     <row r="90" spans="1:20" s="28" customFormat="1" ht="39.950000000000003" customHeight="1">
       <c r="A90" s="25" t="s">
         <v>51</v>
       </c>
       <c r="B90" s="25"/>
-      <c r="C90" s="80" t="s">
+      <c r="C90" s="87" t="s">
         <v>111</v>
       </c>
-      <c r="D90" s="80"/>
-      <c r="E90" s="80"/>
-      <c r="F90" s="80"/>
-      <c r="G90" s="80"/>
-      <c r="H90" s="80"/>
-      <c r="I90" s="80"/>
-      <c r="J90" s="80"/>
-      <c r="K90" s="80"/>
-      <c r="L90" s="80"/>
+      <c r="D90" s="87"/>
+      <c r="E90" s="87"/>
+      <c r="F90" s="87"/>
+      <c r="G90" s="87"/>
+      <c r="H90" s="87"/>
+      <c r="I90" s="87"/>
+      <c r="J90" s="87"/>
+      <c r="K90" s="87"/>
+      <c r="L90" s="87"/>
     </row>
     <row r="91" spans="1:20" s="28" customFormat="1" ht="30" customHeight="1">
-      <c r="A91" s="78" t="s">
+      <c r="A91" s="84" t="s">
         <v>112</v>
       </c>
-      <c r="B91" s="78"/>
-      <c r="C91" s="78"/>
-      <c r="D91" s="78"/>
-      <c r="E91" s="78"/>
-      <c r="F91" s="78"/>
-      <c r="G91" s="78"/>
-      <c r="H91" s="78"/>
-      <c r="I91" s="78"/>
-      <c r="J91" s="78"/>
-      <c r="K91" s="78"/>
-      <c r="L91" s="78"/>
+      <c r="B91" s="84"/>
+      <c r="C91" s="84"/>
+      <c r="D91" s="84"/>
+      <c r="E91" s="84"/>
+      <c r="F91" s="84"/>
+      <c r="G91" s="84"/>
+      <c r="H91" s="84"/>
+      <c r="I91" s="84"/>
+      <c r="J91" s="84"/>
+      <c r="K91" s="84"/>
+      <c r="L91" s="84"/>
     </row>
     <row r="92" spans="1:20" s="28" customFormat="1" ht="39.950000000000003" customHeight="1">
       <c r="A92" s="25" t="s">
         <v>49</v>
       </c>
       <c r="B92" s="25"/>
-      <c r="C92" s="79" t="s">
+      <c r="C92" s="85" t="s">
         <v>113</v>
       </c>
-      <c r="D92" s="79"/>
-      <c r="E92" s="79"/>
-      <c r="F92" s="79"/>
-      <c r="G92" s="79"/>
-      <c r="H92" s="79"/>
-      <c r="I92" s="79"/>
-      <c r="J92" s="79"/>
-      <c r="K92" s="79"/>
-      <c r="L92" s="79"/>
+      <c r="D92" s="85"/>
+      <c r="E92" s="85"/>
+      <c r="F92" s="85"/>
+      <c r="G92" s="85"/>
+      <c r="H92" s="85"/>
+      <c r="I92" s="85"/>
+      <c r="J92" s="85"/>
+      <c r="K92" s="85"/>
+      <c r="L92" s="85"/>
     </row>
     <row r="93" spans="1:20" s="28" customFormat="1" ht="39.950000000000003" customHeight="1">
-      <c r="A93" s="79" t="s">
+      <c r="A93" s="85" t="s">
         <v>50</v>
       </c>
-      <c r="B93" s="79"/>
-      <c r="C93" s="80" t="s">
+      <c r="B93" s="85"/>
+      <c r="C93" s="87" t="s">
         <v>114</v>
       </c>
-      <c r="D93" s="80"/>
-      <c r="E93" s="80"/>
-      <c r="F93" s="80"/>
-      <c r="G93" s="80"/>
-      <c r="H93" s="80"/>
-      <c r="I93" s="80"/>
-      <c r="J93" s="80"/>
-      <c r="K93" s="80"/>
-      <c r="L93" s="80"/>
+      <c r="D93" s="87"/>
+      <c r="E93" s="87"/>
+      <c r="F93" s="87"/>
+      <c r="G93" s="87"/>
+      <c r="H93" s="87"/>
+      <c r="I93" s="87"/>
+      <c r="J93" s="87"/>
+      <c r="K93" s="87"/>
+      <c r="L93" s="87"/>
     </row>
     <row r="94" spans="1:20" s="28" customFormat="1" ht="39.950000000000003" customHeight="1">
       <c r="A94" s="25" t="s">
         <v>51</v>
       </c>
       <c r="B94" s="25"/>
-      <c r="C94" s="81" t="s">
+      <c r="C94" s="78" t="s">
         <v>78</v>
       </c>
-      <c r="D94" s="81"/>
-      <c r="E94" s="81"/>
-      <c r="F94" s="81"/>
-      <c r="G94" s="81"/>
-      <c r="H94" s="81"/>
-      <c r="I94" s="81"/>
-      <c r="J94" s="81"/>
-      <c r="K94" s="81"/>
-      <c r="L94" s="81"/>
+      <c r="D94" s="78"/>
+      <c r="E94" s="78"/>
+      <c r="F94" s="78"/>
+      <c r="G94" s="78"/>
+      <c r="H94" s="78"/>
+      <c r="I94" s="78"/>
+      <c r="J94" s="78"/>
+      <c r="K94" s="78"/>
+      <c r="L94" s="78"/>
     </row>
     <row r="95" spans="1:20" s="28" customFormat="1" ht="30" customHeight="1">
-      <c r="A95" s="78" t="s">
+      <c r="A95" s="84" t="s">
         <v>115</v>
       </c>
-      <c r="B95" s="78"/>
-      <c r="C95" s="78"/>
-      <c r="D95" s="78"/>
-      <c r="E95" s="78"/>
-      <c r="F95" s="78"/>
-      <c r="G95" s="78"/>
-      <c r="H95" s="78"/>
-      <c r="I95" s="78"/>
-      <c r="J95" s="78"/>
-      <c r="K95" s="78"/>
-      <c r="L95" s="78"/>
+      <c r="B95" s="84"/>
+      <c r="C95" s="84"/>
+      <c r="D95" s="84"/>
+      <c r="E95" s="84"/>
+      <c r="F95" s="84"/>
+      <c r="G95" s="84"/>
+      <c r="H95" s="84"/>
+      <c r="I95" s="84"/>
+      <c r="J95" s="84"/>
+      <c r="K95" s="84"/>
+      <c r="L95" s="84"/>
     </row>
     <row r="96" spans="1:20" s="28" customFormat="1" ht="39.950000000000003" customHeight="1">
       <c r="A96" s="25" t="s">
         <v>49</v>
       </c>
       <c r="B96" s="25"/>
-      <c r="C96" s="79" t="s">
+      <c r="C96" s="85" t="s">
         <v>116</v>
       </c>
-      <c r="D96" s="79"/>
-      <c r="E96" s="79"/>
-      <c r="F96" s="79"/>
-      <c r="G96" s="79"/>
-      <c r="H96" s="79"/>
-      <c r="I96" s="79"/>
-      <c r="J96" s="79"/>
-      <c r="K96" s="79"/>
-      <c r="L96" s="79"/>
+      <c r="D96" s="85"/>
+      <c r="E96" s="85"/>
+      <c r="F96" s="85"/>
+      <c r="G96" s="85"/>
+      <c r="H96" s="85"/>
+      <c r="I96" s="85"/>
+      <c r="J96" s="85"/>
+      <c r="K96" s="85"/>
+      <c r="L96" s="85"/>
     </row>
     <row r="97" spans="1:12" s="28" customFormat="1" ht="39.950000000000003" customHeight="1">
-      <c r="A97" s="79" t="s">
+      <c r="A97" s="85" t="s">
         <v>50</v>
       </c>
-      <c r="B97" s="79"/>
-      <c r="C97" s="80" t="s">
+      <c r="B97" s="85"/>
+      <c r="C97" s="87" t="s">
         <v>117</v>
       </c>
-      <c r="D97" s="80"/>
-      <c r="E97" s="80"/>
-      <c r="F97" s="80"/>
-      <c r="G97" s="80"/>
-      <c r="H97" s="80"/>
-      <c r="I97" s="80"/>
-      <c r="J97" s="80"/>
-      <c r="K97" s="80"/>
-      <c r="L97" s="80"/>
+      <c r="D97" s="87"/>
+      <c r="E97" s="87"/>
+      <c r="F97" s="87"/>
+      <c r="G97" s="87"/>
+      <c r="H97" s="87"/>
+      <c r="I97" s="87"/>
+      <c r="J97" s="87"/>
+      <c r="K97" s="87"/>
+      <c r="L97" s="87"/>
     </row>
     <row r="98" spans="1:12" s="28" customFormat="1" ht="39.950000000000003" customHeight="1">
       <c r="A98" s="25" t="s">
         <v>51</v>
       </c>
       <c r="B98" s="25"/>
-      <c r="C98" s="81" t="s">
+      <c r="C98" s="78" t="s">
         <v>118</v>
       </c>
-      <c r="D98" s="81"/>
-      <c r="E98" s="81"/>
-      <c r="F98" s="81"/>
-      <c r="G98" s="81"/>
-      <c r="H98" s="81"/>
-      <c r="I98" s="81"/>
-      <c r="J98" s="81"/>
-      <c r="K98" s="81"/>
-      <c r="L98" s="81"/>
+      <c r="D98" s="78"/>
+      <c r="E98" s="78"/>
+      <c r="F98" s="78"/>
+      <c r="G98" s="78"/>
+      <c r="H98" s="78"/>
+      <c r="I98" s="78"/>
+      <c r="J98" s="78"/>
+      <c r="K98" s="78"/>
+      <c r="L98" s="78"/>
     </row>
     <row r="99" spans="1:12" ht="21.75" customHeight="1">
       <c r="A99" s="3"/>
@@ -16045,30 +16044,36 @@
     </row>
   </sheetData>
   <mergeCells count="67">
-    <mergeCell ref="C54:L54"/>
-    <mergeCell ref="A2:K2"/>
-    <mergeCell ref="A3:A4"/>
-    <mergeCell ref="B3:E3"/>
-    <mergeCell ref="F3:I3"/>
-    <mergeCell ref="J3:K3"/>
-    <mergeCell ref="A43:L47"/>
-    <mergeCell ref="A50:L50"/>
-    <mergeCell ref="A51:L51"/>
-    <mergeCell ref="B52:L52"/>
-    <mergeCell ref="A53:B53"/>
-    <mergeCell ref="C53:L53"/>
-    <mergeCell ref="C64:L64"/>
-    <mergeCell ref="A55:L55"/>
-    <mergeCell ref="B56:L56"/>
-    <mergeCell ref="A57:B57"/>
-    <mergeCell ref="C57:L57"/>
-    <mergeCell ref="B58:L58"/>
-    <mergeCell ref="A59:L59"/>
-    <mergeCell ref="B60:L60"/>
-    <mergeCell ref="A61:B61"/>
-    <mergeCell ref="C61:L61"/>
-    <mergeCell ref="C62:L62"/>
-    <mergeCell ref="A63:L63"/>
+    <mergeCell ref="A95:L95"/>
+    <mergeCell ref="C96:L96"/>
+    <mergeCell ref="A97:B97"/>
+    <mergeCell ref="C97:L97"/>
+    <mergeCell ref="C98:L98"/>
+    <mergeCell ref="C94:L94"/>
+    <mergeCell ref="A85:B85"/>
+    <mergeCell ref="C85:L85"/>
+    <mergeCell ref="C86:L86"/>
+    <mergeCell ref="A87:L87"/>
+    <mergeCell ref="C88:L88"/>
+    <mergeCell ref="A89:B89"/>
+    <mergeCell ref="C89:L89"/>
+    <mergeCell ref="C90:L90"/>
+    <mergeCell ref="A91:L91"/>
+    <mergeCell ref="C92:L92"/>
+    <mergeCell ref="A93:B93"/>
+    <mergeCell ref="C93:L93"/>
+    <mergeCell ref="C84:L84"/>
+    <mergeCell ref="A75:L75"/>
+    <mergeCell ref="C76:L76"/>
+    <mergeCell ref="A77:B77"/>
+    <mergeCell ref="C77:L77"/>
+    <mergeCell ref="C78:L78"/>
+    <mergeCell ref="A79:L79"/>
+    <mergeCell ref="C80:L80"/>
+    <mergeCell ref="A81:B81"/>
+    <mergeCell ref="C81:L81"/>
+    <mergeCell ref="C82:L82"/>
+    <mergeCell ref="A83:L83"/>
     <mergeCell ref="C74:L74"/>
     <mergeCell ref="A65:B65"/>
     <mergeCell ref="C65:L65"/>
@@ -16082,36 +16087,30 @@
     <mergeCell ref="C72:L72"/>
     <mergeCell ref="A73:B73"/>
     <mergeCell ref="C73:L73"/>
-    <mergeCell ref="C84:L84"/>
-    <mergeCell ref="A75:L75"/>
-    <mergeCell ref="C76:L76"/>
-    <mergeCell ref="A77:B77"/>
-    <mergeCell ref="C77:L77"/>
-    <mergeCell ref="C78:L78"/>
-    <mergeCell ref="A79:L79"/>
-    <mergeCell ref="C80:L80"/>
-    <mergeCell ref="A81:B81"/>
-    <mergeCell ref="C81:L81"/>
-    <mergeCell ref="C82:L82"/>
-    <mergeCell ref="A83:L83"/>
-    <mergeCell ref="C94:L94"/>
-    <mergeCell ref="A85:B85"/>
-    <mergeCell ref="C85:L85"/>
-    <mergeCell ref="C86:L86"/>
-    <mergeCell ref="A87:L87"/>
-    <mergeCell ref="C88:L88"/>
-    <mergeCell ref="A89:B89"/>
-    <mergeCell ref="C89:L89"/>
-    <mergeCell ref="C90:L90"/>
-    <mergeCell ref="A91:L91"/>
-    <mergeCell ref="C92:L92"/>
-    <mergeCell ref="A93:B93"/>
-    <mergeCell ref="C93:L93"/>
-    <mergeCell ref="A95:L95"/>
-    <mergeCell ref="C96:L96"/>
-    <mergeCell ref="A97:B97"/>
-    <mergeCell ref="C97:L97"/>
-    <mergeCell ref="C98:L98"/>
+    <mergeCell ref="C64:L64"/>
+    <mergeCell ref="A55:L55"/>
+    <mergeCell ref="B56:L56"/>
+    <mergeCell ref="A57:B57"/>
+    <mergeCell ref="C57:L57"/>
+    <mergeCell ref="B58:L58"/>
+    <mergeCell ref="A59:L59"/>
+    <mergeCell ref="B60:L60"/>
+    <mergeCell ref="A61:B61"/>
+    <mergeCell ref="C61:L61"/>
+    <mergeCell ref="C62:L62"/>
+    <mergeCell ref="A63:L63"/>
+    <mergeCell ref="C54:L54"/>
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="A3:A4"/>
+    <mergeCell ref="B3:E3"/>
+    <mergeCell ref="F3:I3"/>
+    <mergeCell ref="J3:K3"/>
+    <mergeCell ref="A43:L47"/>
+    <mergeCell ref="A50:L50"/>
+    <mergeCell ref="A51:L51"/>
+    <mergeCell ref="B52:L52"/>
+    <mergeCell ref="A53:B53"/>
+    <mergeCell ref="C53:L53"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>